<commit_message>
chore: update repository files
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\musny\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\musny\Desktop\GPA_Cal\result_backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{772126D5-C53E-4EB2-B16B-E2894A52CD65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA2D0336-AF6C-4B99-AB16-6B9AAEF3F8B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4398,7 +4398,7 @@
         <v>236</v>
       </c>
       <c r="H99" s="4">
-        <f t="shared" ref="H99:H130" si="3">IFERROR(
+        <f t="shared" ref="H99:H108" si="3">IFERROR(
 ROUND(
 (
 (IF(C99="A+", 4, IF(C99="A", 4, IF(C99="A-", 3.7, IF(C99="B+", 3.3, IF(C99="B", 3, IF(C99="B-", 2.7, IF(C99="C+", 2.3, IF(C99="C", 2, IF(C99="C-", 1.7, IF(C99="D+", 1.3, IF(C99="D", 1, IF(C99="E", 0, 0)))))))))))) * 4) +
@@ -12427,7 +12427,7 @@
         <v>244</v>
       </c>
       <c r="H99" s="3">
-        <f t="shared" ref="H99:H130" si="3">IFERROR(
+        <f t="shared" ref="H99:H108" si="3">IFERROR(
 ROUND(
 (
 (IF(C99="A+", 4, IF(C99="A", 4, IF(C99="A-", 3.7, IF(C99="B+", 3.3, IF(C99="B", 3, IF(C99="B-", 2.7, IF(C99="C+", 2.3, IF(C99="C", 2, IF(C99="C-", 1.7, IF(C99="D+", 1.3, IF(C99="D", 1, IF(C99="E", 0, 0))))))))))))) * 4 +
@@ -20447,7 +20447,7 @@
         <v>236</v>
       </c>
       <c r="I99" s="3">
-        <f t="shared" ref="I99:I130" si="3">IFERROR(
+        <f t="shared" ref="I99:I108" si="3">IFERROR(
 ROUND(
 (
 (IF(C99="A+", 4, IF(C99="A", 4, IF(C99="A-", 3.7, IF(C99="B+", 3.3, IF(C99="B", 3, IF(C99="B-", 2.7, IF(C99="C+", 2.3, IF(C99="C", 2, IF(C99="C-", 1.7, IF(C99="D+", 1.3, IF(C99="D", 1, IF(C99="E", 0, 0))))))))))))) * 3 +
@@ -21886,7 +21886,7 @@
         <v>236</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>253</v>
+        <v>244</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>238</v>
@@ -21902,7 +21902,7 @@
       </c>
       <c r="I8" s="3">
         <f t="shared" si="0"/>
-        <v>2.61</v>
+        <v>3.01</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
@@ -24655,7 +24655,7 @@
         <v>242</v>
       </c>
       <c r="I99" s="3">
-        <f t="shared" ref="I99:I130" si="3">IFERROR(
+        <f t="shared" ref="I99:I108" si="3">IFERROR(
 ROUND(
 (
 (IF(C99="A+", 4, IF(C99="A", 4, IF(C99="A-", 3.7, IF(C99="B+", 3.3, IF(C99="B", 3, IF(C99="B-", 2.7, IF(C99="C+", 2.3, IF(C99="C", 2, IF(C99="C-", 1.7, IF(C99="D+", 1.3, IF(C99="D", 1, IF(C99="E", 0, 0))))))))))))) * 3 +
@@ -24742,7 +24742,7 @@
         <v>236</v>
       </c>
       <c r="D102" s="3" t="s">
-        <v>252</v>
+        <v>239</v>
       </c>
       <c r="E102" s="22" t="s">
         <v>237</v>
@@ -24758,7 +24758,7 @@
       </c>
       <c r="I102" s="3">
         <f t="shared" si="3"/>
-        <v>2.74</v>
+        <v>2.88</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
@@ -28471,11 +28471,11 @@
         <v>2.75</v>
       </c>
       <c r="H8" s="27">
-        <v>2.61</v>
+        <v>3.01</v>
       </c>
       <c r="I8" s="29">
         <f t="shared" si="0"/>
-        <v>2.6280000000000001</v>
+        <v>2.6949999999999998</v>
       </c>
       <c r="J8" s="29" t="str">
         <f>IFERROR(VLOOKUP(A8, '4.1'!$A$2:$O$52, 15, FALSE), "N/A")</f>
@@ -28491,7 +28491,7 @@
       </c>
       <c r="M8" s="29">
         <f t="shared" si="2"/>
-        <v>2.6280000000000001</v>
+        <v>2.6949999999999998</v>
       </c>
       <c r="N8" s="29" t="str">
         <f t="shared" si="3"/>
@@ -33514,7 +33514,7 @@
         <v>3.58</v>
       </c>
       <c r="I98" s="29">
-        <f t="shared" ref="I98:I129" si="15">ROUND(AVERAGE(C98:H98), 3)</f>
+        <f t="shared" ref="I98:I108" si="15">ROUND(AVERAGE(C98:H98), 3)</f>
         <v>3.2919999999999998</v>
       </c>
       <c r="J98" s="29">
@@ -33526,11 +33526,11 @@
         <v>4</v>
       </c>
       <c r="L98" s="29">
-        <f t="shared" ref="L98:L129" si="16">IF(ISNUMBER(J98), ROUND((J98*24 + K98*6)/30, 3), "N/A")</f>
+        <f t="shared" ref="L98:L108" si="16">IF(ISNUMBER(J98), ROUND((J98*24 + K98*6)/30, 3), "N/A")</f>
         <v>3.7519999999999998</v>
       </c>
       <c r="M98" s="29">
-        <f t="shared" ref="M98:M129" si="17">IF(ISNUMBER(L98), ROUND(I98*0.75 + L98*0.25, 3), I98)</f>
+        <f t="shared" ref="M98:M108" si="17">IF(ISNUMBER(L98), ROUND(I98*0.75 + L98*0.25, 3), I98)</f>
         <v>3.407</v>
       </c>
       <c r="N98" s="29" t="str">
@@ -33735,11 +33735,11 @@
         <v>3.29</v>
       </c>
       <c r="H102" s="27">
-        <v>2.74</v>
+        <v>2.88</v>
       </c>
       <c r="I102" s="29">
         <f t="shared" si="15"/>
-        <v>2.802</v>
+        <v>2.8250000000000002</v>
       </c>
       <c r="J102" s="29" t="str">
         <f>IFERROR(VLOOKUP(A102, '4.1'!$A$2:$O$52, 15, FALSE), "N/A")</f>
@@ -33755,7 +33755,7 @@
       </c>
       <c r="M102" s="29">
         <f t="shared" si="17"/>
-        <v>2.802</v>
+        <v>2.8250000000000002</v>
       </c>
       <c r="N102" s="29" t="str">
         <f t="shared" si="18"/>

</xml_diff>